<commit_message>
code of experiments updated
</commit_message>
<xml_diff>
--- a/experimental_results/Supplementary experimental results.xlsx
+++ b/experimental_results/Supplementary experimental results.xlsx
@@ -5,27 +5,41 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\新建文件夹\VPP\会议\icassp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SDC\xwechat_files\wxid_iebtrz3mce8e22_eff4\msg\file\2025-12\FMDST\FMDST\experimental_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2833C1-B96E-4545-93A7-1703609D824E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3811FCD-2595-4E9E-8F6E-DF82738EE220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Main_Results_After_Review" sheetId="1" r:id="rId1"/>
+    <sheet name="Horizon_Comparison_2h" sheetId="2" r:id="rId2"/>
+    <sheet name="Horizon_Comparison_3h" sheetId="3" r:id="rId3"/>
+    <sheet name="Horizon_Comparison_10h" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="33">
   <si>
     <t>LSTM</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -132,6 +146,29 @@
   </si>
   <si>
     <t>LSTM (1 hours)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Experimental results for 2 hours MAE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ST_ReP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">                                       Average_MAE</t>
+  </si>
+  <si>
+    <t>Experimental results for 3 hours MAE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">                                       Average_MAE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Experimental results for 10 hours MAE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -139,7 +176,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -163,8 +200,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -174,6 +219,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -190,9 +241,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1299,4 +1352,1180 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3DCC912-7869-455F-A756-5E757F34051E}">
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.08203125" customWidth="1"/>
+    <col min="3" max="3" width="15.08203125" customWidth="1"/>
+    <col min="4" max="4" width="17.08203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>52.346699999999998</v>
+      </c>
+      <c r="C3">
+        <v>60.360900000000001</v>
+      </c>
+      <c r="D3">
+        <v>72.416799999999995</v>
+      </c>
+      <c r="E3">
+        <v>52.606900000000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>70.308400000000006</v>
+      </c>
+      <c r="C4">
+        <v>72.290400000000005</v>
+      </c>
+      <c r="D4">
+        <v>80.212000000000003</v>
+      </c>
+      <c r="E4">
+        <v>65.315600000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>81.403899999999993</v>
+      </c>
+      <c r="C5">
+        <v>87.446100000000001</v>
+      </c>
+      <c r="D5">
+        <v>87.777900000000002</v>
+      </c>
+      <c r="E5">
+        <v>75.419300000000007</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>90.409800000000004</v>
+      </c>
+      <c r="C6">
+        <v>94.372399999999999</v>
+      </c>
+      <c r="D6">
+        <v>95.059399999999997</v>
+      </c>
+      <c r="E6">
+        <v>84.553600000000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>98.973799999999997</v>
+      </c>
+      <c r="C7">
+        <v>101.8873</v>
+      </c>
+      <c r="D7">
+        <v>101.8175</v>
+      </c>
+      <c r="E7">
+        <v>92.508700000000005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>107.32</v>
+      </c>
+      <c r="C8">
+        <v>110.6571</v>
+      </c>
+      <c r="D8">
+        <v>107.9611</v>
+      </c>
+      <c r="E8">
+        <v>101.4101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>115.298</v>
+      </c>
+      <c r="C9">
+        <v>117.5697</v>
+      </c>
+      <c r="D9">
+        <v>113.6833</v>
+      </c>
+      <c r="E9">
+        <v>109.17870000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>121.0848</v>
+      </c>
+      <c r="C10">
+        <v>121.9406</v>
+      </c>
+      <c r="D10">
+        <v>119.1568</v>
+      </c>
+      <c r="E10">
+        <v>115.2595</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>125.84820000000001</v>
+      </c>
+      <c r="C11">
+        <v>128.39699999999999</v>
+      </c>
+      <c r="D11">
+        <v>124.5124</v>
+      </c>
+      <c r="E11">
+        <v>122.28189999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>134.96449999999999</v>
+      </c>
+      <c r="C12">
+        <v>134.96369999999999</v>
+      </c>
+      <c r="D12">
+        <v>129.4699</v>
+      </c>
+      <c r="E12">
+        <v>129.54740000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>140.02590000000001</v>
+      </c>
+      <c r="C13">
+        <v>142.3014</v>
+      </c>
+      <c r="D13">
+        <v>134.2664</v>
+      </c>
+      <c r="E13">
+        <v>136.73939999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>144.893</v>
+      </c>
+      <c r="C14">
+        <v>145.1772</v>
+      </c>
+      <c r="D14">
+        <v>138.74350000000001</v>
+      </c>
+      <c r="E14">
+        <v>142.51230000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15">
+        <v>106.9064</v>
+      </c>
+      <c r="C15">
+        <v>109.7803</v>
+      </c>
+      <c r="D15">
+        <v>108.7564</v>
+      </c>
+      <c r="E15">
+        <v>102.2778</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D0EDE20-78AF-455B-A544-A23FC222EE26}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="33.9140625" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.08203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>54.253100000000003</v>
+      </c>
+      <c r="C3">
+        <v>62.302399999999999</v>
+      </c>
+      <c r="D3">
+        <v>60.996499999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>71.197900000000004</v>
+      </c>
+      <c r="C4">
+        <v>73.195599999999999</v>
+      </c>
+      <c r="D4">
+        <v>72.352500000000006</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>82.895499999999998</v>
+      </c>
+      <c r="C5">
+        <v>86.190399999999997</v>
+      </c>
+      <c r="D5">
+        <v>82.139899999999997</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>92.048500000000004</v>
+      </c>
+      <c r="C6">
+        <v>97.396699999999996</v>
+      </c>
+      <c r="D6">
+        <v>90.246300000000005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>100.4042</v>
+      </c>
+      <c r="C7">
+        <v>100.8032</v>
+      </c>
+      <c r="D7">
+        <v>97.889200000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>108.4414</v>
+      </c>
+      <c r="C8">
+        <v>110.89879999999999</v>
+      </c>
+      <c r="D8">
+        <v>106.12090000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>115.0673</v>
+      </c>
+      <c r="C9">
+        <v>121.6352</v>
+      </c>
+      <c r="D9">
+        <v>113.94580000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>122.2895</v>
+      </c>
+      <c r="C10">
+        <v>127.6666</v>
+      </c>
+      <c r="D10">
+        <v>120.5382</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>129.059</v>
+      </c>
+      <c r="C11">
+        <v>133.369</v>
+      </c>
+      <c r="D11">
+        <v>127.0818</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>135.26779999999999</v>
+      </c>
+      <c r="C12">
+        <v>139.64179999999999</v>
+      </c>
+      <c r="D12">
+        <v>134.05369999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>142.4435</v>
+      </c>
+      <c r="C13">
+        <v>144.02930000000001</v>
+      </c>
+      <c r="D13">
+        <v>140.69579999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>147.29239999999999</v>
+      </c>
+      <c r="C14">
+        <v>148.76929999999999</v>
+      </c>
+      <c r="D14">
+        <v>146.21709999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>151.16460000000001</v>
+      </c>
+      <c r="C15">
+        <v>152.2723</v>
+      </c>
+      <c r="D15">
+        <v>150.88929999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>157.00700000000001</v>
+      </c>
+      <c r="C16">
+        <v>156.4726</v>
+      </c>
+      <c r="D16">
+        <v>156.77260000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <v>162.68780000000001</v>
+      </c>
+      <c r="C17">
+        <v>164.2585</v>
+      </c>
+      <c r="D17">
+        <v>162.26669999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <v>170.02930000000001</v>
+      </c>
+      <c r="C18">
+        <v>169.67320000000001</v>
+      </c>
+      <c r="D18">
+        <v>168.32660000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B19">
+        <v>173.50200000000001</v>
+      </c>
+      <c r="C19">
+        <v>172.09059999999999</v>
+      </c>
+      <c r="D19">
+        <v>173.09059999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <v>178.10740000000001</v>
+      </c>
+      <c r="C20">
+        <v>179.51499999999999</v>
+      </c>
+      <c r="D20">
+        <v>178.27109999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21">
+        <v>127.79770000000001</v>
+      </c>
+      <c r="C21">
+        <v>130.01</v>
+      </c>
+      <c r="D21">
+        <v>126.77200000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C9880F1-BAD8-43F0-B318-7DC3A1871E6C}">
+  <dimension ref="A1:D63"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="34.08203125" customWidth="1"/>
+    <col min="2" max="2" width="12.9140625" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" customWidth="1"/>
+    <col min="4" max="4" width="13.58203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="3"/>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>71.331800000000001</v>
+      </c>
+      <c r="C3">
+        <v>101.06359999999999</v>
+      </c>
+      <c r="D3">
+        <v>106.09690000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>83.825699999999998</v>
+      </c>
+      <c r="C4">
+        <v>119.693</v>
+      </c>
+      <c r="D4">
+        <v>113.11969999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>94.544399999999996</v>
+      </c>
+      <c r="C5">
+        <v>113.4008</v>
+      </c>
+      <c r="D5">
+        <v>120.1138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>104.6833</v>
+      </c>
+      <c r="C6">
+        <v>135.9135</v>
+      </c>
+      <c r="D6">
+        <v>126.22029999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <v>114.04989999999999</v>
+      </c>
+      <c r="C7">
+        <v>134.75</v>
+      </c>
+      <c r="D7">
+        <v>132.53200000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <v>119.569</v>
+      </c>
+      <c r="C8">
+        <v>139.57550000000001</v>
+      </c>
+      <c r="D8">
+        <v>137.6858</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>126.6435</v>
+      </c>
+      <c r="C9">
+        <v>148.0909</v>
+      </c>
+      <c r="D9">
+        <v>143.29570000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <v>135.13149999999999</v>
+      </c>
+      <c r="C10">
+        <v>144.10120000000001</v>
+      </c>
+      <c r="D10">
+        <v>149.4803</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B11">
+        <v>144.63399999999999</v>
+      </c>
+      <c r="C11">
+        <v>150.20480000000001</v>
+      </c>
+      <c r="D11">
+        <v>155.11750000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12">
+        <v>150.07579999999999</v>
+      </c>
+      <c r="C12">
+        <v>152.3974</v>
+      </c>
+      <c r="D12">
+        <v>159.44370000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B13">
+        <v>156.20269999999999</v>
+      </c>
+      <c r="C13">
+        <v>159.7396</v>
+      </c>
+      <c r="D13">
+        <v>164.1857</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B14">
+        <v>159.52180000000001</v>
+      </c>
+      <c r="C14">
+        <v>165.7158</v>
+      </c>
+      <c r="D14">
+        <v>169.12260000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B15">
+        <v>166.33600000000001</v>
+      </c>
+      <c r="C15">
+        <v>178.2456</v>
+      </c>
+      <c r="D15">
+        <v>173.2226</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16">
+        <v>171.95099999999999</v>
+      </c>
+      <c r="C16">
+        <v>171.18719999999999</v>
+      </c>
+      <c r="D16">
+        <v>176.52170000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17">
+        <v>174.9648</v>
+      </c>
+      <c r="C17">
+        <v>178.43020000000001</v>
+      </c>
+      <c r="D17">
+        <v>178.62119999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B18">
+        <v>177.95339999999999</v>
+      </c>
+      <c r="C18">
+        <v>178.06399999999999</v>
+      </c>
+      <c r="D18">
+        <v>180.99700000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B19">
+        <v>184.18559999999999</v>
+      </c>
+      <c r="C19">
+        <v>181.78960000000001</v>
+      </c>
+      <c r="D19">
+        <v>185.3245</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20">
+        <v>188.88310000000001</v>
+      </c>
+      <c r="C20">
+        <v>189.10419999999999</v>
+      </c>
+      <c r="D20">
+        <v>188.41399999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B21">
+        <v>195.0909</v>
+      </c>
+      <c r="C21">
+        <v>195.7792</v>
+      </c>
+      <c r="D21">
+        <v>191.76130000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B22">
+        <v>198.51419999999999</v>
+      </c>
+      <c r="C22">
+        <v>195.93379999999999</v>
+      </c>
+      <c r="D22">
+        <v>195.6737</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B23">
+        <v>205.4366</v>
+      </c>
+      <c r="C23">
+        <v>210.0556</v>
+      </c>
+      <c r="D23">
+        <v>200.85900000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B24">
+        <v>206.19990000000001</v>
+      </c>
+      <c r="C24">
+        <v>206.7739</v>
+      </c>
+      <c r="D24">
+        <v>204.87739999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B25">
+        <v>213.2927</v>
+      </c>
+      <c r="C25">
+        <v>217.92019999999999</v>
+      </c>
+      <c r="D25">
+        <v>208.78710000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B26">
+        <v>217.49940000000001</v>
+      </c>
+      <c r="C26">
+        <v>223.47329999999999</v>
+      </c>
+      <c r="D26">
+        <v>213.1241</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B27">
+        <v>220.6439</v>
+      </c>
+      <c r="C27">
+        <v>221.97470000000001</v>
+      </c>
+      <c r="D27">
+        <v>215.3468</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B28">
+        <v>222.26410000000001</v>
+      </c>
+      <c r="C28">
+        <v>228.77</v>
+      </c>
+      <c r="D28">
+        <v>218.61940000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B29">
+        <v>227.44120000000001</v>
+      </c>
+      <c r="C29">
+        <v>235.40889999999999</v>
+      </c>
+      <c r="D29">
+        <v>222.4836</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B30">
+        <v>229.8733</v>
+      </c>
+      <c r="C30">
+        <v>238.45089999999999</v>
+      </c>
+      <c r="D30">
+        <v>224.9495</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B31">
+        <v>235.78</v>
+      </c>
+      <c r="C31">
+        <v>238.11879999999999</v>
+      </c>
+      <c r="D31">
+        <v>228.88130000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>239.0119</v>
+      </c>
+      <c r="C32">
+        <v>245.54769999999999</v>
+      </c>
+      <c r="D32">
+        <v>233.0224</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B33">
+        <v>243.95099999999999</v>
+      </c>
+      <c r="C33">
+        <v>249.2843</v>
+      </c>
+      <c r="D33">
+        <v>236.33930000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B34">
+        <v>245.61420000000001</v>
+      </c>
+      <c r="C34">
+        <v>246.62039999999999</v>
+      </c>
+      <c r="D34">
+        <v>239.94069999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B35">
+        <v>250.7346</v>
+      </c>
+      <c r="C35">
+        <v>253.58629999999999</v>
+      </c>
+      <c r="D35">
+        <v>242.4864</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B36">
+        <v>253.7209</v>
+      </c>
+      <c r="C36">
+        <v>254.72069999999999</v>
+      </c>
+      <c r="D36">
+        <v>245.98249999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B37">
+        <v>255.87610000000001</v>
+      </c>
+      <c r="C37">
+        <v>256.84570000000002</v>
+      </c>
+      <c r="D37">
+        <v>249.57509999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B38">
+        <v>260.3605</v>
+      </c>
+      <c r="C38">
+        <v>261.18239999999997</v>
+      </c>
+      <c r="D38">
+        <v>252.9598</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B39">
+        <v>265.56740000000002</v>
+      </c>
+      <c r="C39">
+        <v>274.71289999999999</v>
+      </c>
+      <c r="D39">
+        <v>256.38619999999997</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B40">
+        <v>267.43239999999997</v>
+      </c>
+      <c r="C40">
+        <v>270.75349999999997</v>
+      </c>
+      <c r="D40">
+        <v>259.7432</v>
+      </c>
+    </row>
+    <row r="41" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B41">
+        <v>266.87479999999999</v>
+      </c>
+      <c r="C41">
+        <v>274.67529999999999</v>
+      </c>
+      <c r="D41">
+        <v>261.96949999999998</v>
+      </c>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B42">
+        <v>271.67090000000002</v>
+      </c>
+      <c r="C42">
+        <v>277.72899999999998</v>
+      </c>
+      <c r="D42">
+        <v>265.27089999999998</v>
+      </c>
+    </row>
+    <row r="43" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B43">
+        <v>274.4221</v>
+      </c>
+      <c r="C43">
+        <v>280.36320000000001</v>
+      </c>
+      <c r="D43">
+        <v>269.1782</v>
+      </c>
+    </row>
+    <row r="44" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B44">
+        <v>279.73930000000001</v>
+      </c>
+      <c r="C44">
+        <v>285.947</v>
+      </c>
+      <c r="D44">
+        <v>273.07619999999997</v>
+      </c>
+    </row>
+    <row r="45" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B45">
+        <v>284.9701</v>
+      </c>
+      <c r="C45">
+        <v>293.80410000000001</v>
+      </c>
+      <c r="D45">
+        <v>276.2724</v>
+      </c>
+    </row>
+    <row r="46" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B46">
+        <v>285.60480000000001</v>
+      </c>
+      <c r="C46">
+        <v>291.45</v>
+      </c>
+      <c r="D46">
+        <v>277.98989999999998</v>
+      </c>
+    </row>
+    <row r="47" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B47">
+        <v>290.09640000000002</v>
+      </c>
+      <c r="C47">
+        <v>295.86680000000001</v>
+      </c>
+      <c r="D47">
+        <v>282.64249999999998</v>
+      </c>
+    </row>
+    <row r="48" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B48">
+        <v>291.19319999999999</v>
+      </c>
+      <c r="C48">
+        <v>303.947</v>
+      </c>
+      <c r="D48">
+        <v>284.464</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B49">
+        <v>293.97329999999999</v>
+      </c>
+      <c r="C49">
+        <v>305.7509</v>
+      </c>
+      <c r="D49">
+        <v>286.39299999999997</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B50">
+        <v>294.24029999999999</v>
+      </c>
+      <c r="C50">
+        <v>302.68</v>
+      </c>
+      <c r="D50">
+        <v>289.45839999999998</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B51">
+        <v>298.01299999999998</v>
+      </c>
+      <c r="C51">
+        <v>312.28890000000001</v>
+      </c>
+      <c r="D51">
+        <v>293.15089999999998</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B52">
+        <v>301.53300000000002</v>
+      </c>
+      <c r="C52">
+        <v>310.2876</v>
+      </c>
+      <c r="D52">
+        <v>295.34140000000002</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B53">
+        <v>302.09550000000002</v>
+      </c>
+      <c r="C53">
+        <v>313.50670000000002</v>
+      </c>
+      <c r="D53">
+        <v>297.435</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B54">
+        <v>306.37830000000002</v>
+      </c>
+      <c r="C54">
+        <v>313.14350000000002</v>
+      </c>
+      <c r="D54">
+        <v>300.48390000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B55">
+        <v>309.70940000000002</v>
+      </c>
+      <c r="C55">
+        <v>316.91340000000002</v>
+      </c>
+      <c r="D55">
+        <v>302.83350000000002</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B56">
+        <v>307.935</v>
+      </c>
+      <c r="C56">
+        <v>324.07670000000002</v>
+      </c>
+      <c r="D56">
+        <v>305.11099999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B57">
+        <v>312.49009999999998</v>
+      </c>
+      <c r="C57">
+        <v>323.18849999999998</v>
+      </c>
+      <c r="D57">
+        <v>307.82170000000002</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B58">
+        <v>314.10390000000001</v>
+      </c>
+      <c r="C58">
+        <v>324.3861</v>
+      </c>
+      <c r="D58">
+        <v>309.52109999999999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B59">
+        <v>315.34649999999999</v>
+      </c>
+      <c r="C59">
+        <v>328.03370000000001</v>
+      </c>
+      <c r="D59">
+        <v>312.08080000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B60">
+        <v>316.64940000000001</v>
+      </c>
+      <c r="C60">
+        <v>337.24650000000003</v>
+      </c>
+      <c r="D60">
+        <v>313.7081</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B61">
+        <v>319.2765</v>
+      </c>
+      <c r="C61">
+        <v>336.73700000000002</v>
+      </c>
+      <c r="D61">
+        <v>315.7525</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B62">
+        <v>319.08370000000002</v>
+      </c>
+      <c r="C62">
+        <v>338.38029999999998</v>
+      </c>
+      <c r="D62">
+        <v>317.76</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B63">
+        <v>228.9032</v>
+      </c>
+      <c r="C63">
+        <v>237.62970000000001</v>
+      </c>
+      <c r="D63">
+        <v>228.9838</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>